<commit_message>
feat: NDT 규격 DB 고도화 (ASME, KS, ISO, AWS 판정 기준 및 ASTM 장비 자재 요건 통합)
</commit_message>
<xml_diff>
--- a/home/src/Daily_Economic_Report_20260715.xlsx
+++ b/home/src/Daily_Economic_Report_20260715.xlsx
@@ -450,10 +450,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>7350.81</v>
+        <v>7284.41</v>
       </c>
       <c r="C2" t="n">
-        <v>7.99</v>
+        <v>7.01</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -468,14 +468,14 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>26107.01</v>
+        <v>26143.62</v>
       </c>
       <c r="C3" t="n">
-        <v>0.9</v>
+        <v>1.05</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
     </row>
@@ -486,14 +486,14 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7543.59</v>
+        <v>7553.44</v>
       </c>
       <c r="C4" t="n">
-        <v>0.38</v>
+        <v>0.51</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
     </row>
@@ -504,10 +504,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1490.58</v>
+        <v>1491.63</v>
       </c>
       <c r="C5" t="n">
-        <v>-0.48</v>
+        <v>-0.41</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -522,14 +522,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>80.27</v>
+        <v>79.29000000000001</v>
       </c>
       <c r="C6" t="n">
-        <v>2.73</v>
+        <v>-0.06</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
     </row>
@@ -633,15 +633,15 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>28,000원</t>
+          <t>27,925원</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.32</v>
+        <v>0.05</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>54%</t>
+          <t>150%</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -656,7 +656,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>28,331원</t>
+          <t>28,328원</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -694,15 +694,15 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>196,705원</t>
+          <t>196,500원</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1.12</v>
+        <v>1.01</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>44%</t>
+          <t>87%</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -717,7 +717,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>200,681원</t>
+          <t>200,680원</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -755,20 +755,20 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>15,265원</t>
+          <t>15,210원</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>-1.13</v>
+        <v>-1.49</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>70%</t>
+          <t>136%</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>15,265원</t>
+          <t>15,210원</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -778,7 +778,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>15,556원</t>
+          <t>15,553원</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -816,15 +816,15 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>32,855원</t>
+          <t>32,785원</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>1.28</v>
+        <v>1.06</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>51%</t>
+          <t>96%</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -839,7 +839,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>32,538원</t>
+          <t>32,536원</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -877,15 +877,15 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>61,875원</t>
+          <t>62,200원</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.34</v>
+        <v>2.88</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>51%</t>
+          <t>103%</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>64,564원</t>
+          <t>64,588원</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -946,12 +946,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>35%</t>
+          <t>78%</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>12,420원</t>
+          <t>12,425원</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -999,15 +999,15 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>282,000원</t>
+          <t>279,500원</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>7.22</v>
+        <v>6.27</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>40%</t>
+          <t>81%</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1022,7 +1022,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>311,912원</t>
+          <t>311,850원</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1060,15 +1060,15 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2,143,000원</t>
+          <t>2,082,000원</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>12.02</v>
+        <v>8.83</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>51%</t>
+          <t>101%</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2,422,800원</t>
+          <t>2,420,500원</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1121,15 +1121,15 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>438,500원</t>
+          <t>434,000원</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>3.3</v>
+        <v>2.24</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>47%</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1144,7 +1144,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>495,300원</t>
+          <t>495,075원</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1178,19 +1178,19 @@
         <v>168300</v>
       </c>
       <c r="D11" t="n">
-        <v>6000</v>
+        <v>5400</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>145,600원</t>
+          <t>145,000원</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>4.3</v>
+        <v>3.87</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>45%</t>
+          <t>105%</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1205,7 +1205,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>146,265원</t>
+          <t>146,255원</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1243,15 +1243,15 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>191,400원</t>
+          <t>189,600원</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>4.48</v>
+        <v>3.49</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>31%</t>
+          <t>63%</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1266,7 +1266,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>200,210원</t>
+          <t>200,180원</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1304,15 +1304,15 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1,415,000원</t>
+          <t>1,383,000원</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>3.44</v>
+        <v>1.1</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>64%</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>1,381,950원</t>
+          <t>1,380,450원</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1365,15 +1365,15 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>183,400원</t>
+          <t>181,600원</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>1.89</v>
+        <v>0.89</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>49%</t>
+          <t>105%</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1388,7 +1388,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>165,620원</t>
+          <t>165,505원</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>🚨 전고점 터치 (전량 매도 권장)</t>
+          <t>⚠️ 과열 구간 (분할 매도 준비)</t>
         </is>
       </c>
     </row>
@@ -1426,15 +1426,15 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>$68.76</t>
+          <t>$68.83</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>-0.2</v>
+        <v>-0.09</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>61%</t>
+          <t>11%</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1449,7 +1449,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>$68.35</t>
+          <t>$68.36</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1483,19 +1483,19 @@
         <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$81.51</t>
+          <t>$81.26</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.04</v>
+        <v>-0.26</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>41%</t>
+          <t>58%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1505,17 +1505,17 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>$81.51</t>
+          <t>$81.48</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>$79.27</t>
+          <t>$79.25</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>$77.43</t>
+          <t>$77.41</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1537,26 +1537,26 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>10주</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>6570</v>
+        <v>0</v>
       </c>
       <c r="D17" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>6,830원</t>
+          <t>6,800원</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.25</v>
+        <v>1.8</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>24%</t>
+          <t>33%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1605,19 +1605,19 @@
         <v>5060</v>
       </c>
       <c r="D18" t="n">
-        <v>1400</v>
+        <v>1250</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>4,065원</t>
+          <t>4,050원</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>3.57</v>
+        <v>3.18</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>39%</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1670,15 +1670,15 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>$41.55</t>
+          <t>$40.87</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.04</v>
+        <v>0.37</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>62%</t>
+          <t>23%</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1693,7 +1693,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>$44.22</t>
+          <t>$44.18</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1731,15 +1731,15 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>$79.14</t>
+          <t>$77.00</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>3.76</v>
+        <v>0.96</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>75%</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1754,7 +1754,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>$87.56</t>
+          <t>$87.46</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1792,15 +1792,15 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>$71.58</t>
+          <t>$71.05</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>1.91</v>
+        <v>1.15</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>84%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1815,7 +1815,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>$77.16</t>
+          <t>$77.13</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1830,7 +1830,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>👍 눌림목 매수 (스윙 타점 진입)</t>
+          <t>🔥 패닉 셀링 (과대 낙폭/적극 매수)</t>
         </is>
       </c>
     </row>
@@ -1853,15 +1853,15 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>$78.72</t>
+          <t>$77.52</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>5.88</v>
+        <v>4.26</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>153%</t>
+          <t>13%</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1876,7 +1876,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>$78.89</t>
+          <t>$78.83</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1922,7 +1922,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>38%</t>
+          <t>72%</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>352,675원</t>
+          <t>352,750원</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1975,15 +1975,15 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>462,000원</t>
+          <t>454,000원</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>8.07</v>
+        <v>6.2</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>68%</t>
+          <t>114%</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1998,7 +1998,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>470,150원</t>
+          <t>469,875원</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2032,19 +2032,19 @@
         <v>120000</v>
       </c>
       <c r="D25" t="n">
-        <v>8500</v>
+        <v>8300</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>121,100원</t>
+          <t>120,900원</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>7.55</v>
+        <v>7.37</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>39%</t>
+          <t>66%</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2059,7 +2059,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>135,492원</t>
+          <t>135,500원</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2097,20 +2097,20 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>15,335원</t>
+          <t>15,295원</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>-0.23</v>
+        <v>-0.49</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>14%</t>
+          <t>23%</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>15,335원</t>
+          <t>15,295원</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2120,7 +2120,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>15,688원</t>
+          <t>15,686원</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2158,20 +2158,20 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>13,315원</t>
+          <t>13,275원</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>-0.04</v>
+        <v>-0.34</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>141%</t>
+          <t>179%</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>13,320원</t>
+          <t>13,275원</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2181,7 +2181,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>13,720원</t>
+          <t>13,718원</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2219,15 +2219,15 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>10,120원</t>
+          <t>10,150원</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>46%</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2242,7 +2242,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>10,195원</t>
+          <t>10,196원</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2280,15 +2280,15 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>21,450원</t>
+          <t>21,250원</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>1.66</v>
+        <v>0.71</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>45%</t>
+          <t>115%</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>20,755원</t>
+          <t>20,745원</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2318,7 +2318,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>🚨 전고점 터치 (전량 매도 권장)</t>
+          <t>✅ 보유 (시장 상승세)</t>
         </is>
       </c>
     </row>
@@ -2341,15 +2341,15 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>175,500원</t>
+          <t>172,500원</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>2.63</v>
+        <v>0.88</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>31%</t>
+          <t>111%</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2364,7 +2364,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>174,135원</t>
+          <t>174,000원</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2379,7 +2379,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>✅ 보유 (시장 상승세)</t>
+          <t>🚀 시장 상승 편승 (매수 기회)</t>
         </is>
       </c>
     </row>
@@ -2402,15 +2402,15 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>86,300원</t>
+          <t>85,000원</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>2.86</v>
+        <v>1.31</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>54%</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -2425,7 +2425,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>88,765원</t>
+          <t>88,715원</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2459,19 +2459,19 @@
         <v>217000</v>
       </c>
       <c r="D32" t="n">
-        <v>57500</v>
+        <v>62000</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>265,000원</t>
+          <t>269,500원</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>27.71</v>
+        <v>29.88</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>133%</t>
+          <t>220%</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>246,735원</t>
+          <t>246,985원</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2501,7 +2501,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>✅ 보유 (시장 상승세)</t>
+          <t>🚀 거래량 급증 (수급 폭발)</t>
         </is>
       </c>
     </row>
@@ -2524,15 +2524,15 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1,073,000원</t>
+          <t>1,072,000원</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>0.09</v>
+        <v>0</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>56%</t>
+          <t>98%</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>1,120,550원</t>
+          <t>1,120,250원</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2574,26 +2574,26 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1주</t>
         </is>
       </c>
       <c r="C34" t="n">
         <v>0</v>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>9000</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>279,750원</t>
+          <t>288,500원</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>0.09</v>
+        <v>3.22</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>55%</t>
+          <t>133%</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>338,200원</t>
+          <t>338,600원</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2646,15 +2646,15 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>829,000원</t>
+          <t>823,000원</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>4.02</v>
+        <v>3.26</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>40%</t>
+          <t>82%</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2669,7 +2669,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>923,700원</t>
+          <t>923,400원</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2703,19 +2703,19 @@
         <v>0</v>
       </c>
       <c r="D36" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>35,650원</t>
+          <t>36,500원</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>-2.33</v>
+        <v>0</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>97%</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -2730,7 +2730,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>34,905원</t>
+          <t>34,952원</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2768,15 +2768,15 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>199,900원</t>
+          <t>201,500원</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>6.5</v>
+        <v>7.35</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>44%</t>
+          <t>73%</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2791,7 +2791,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>219,455원</t>
+          <t>219,505원</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2825,19 +2825,19 @@
         <v>1300</v>
       </c>
       <c r="D38" t="n">
-        <v>5000</v>
+        <v>3800</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1,044원</t>
+          <t>1,038원</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>2.45</v>
+        <v>1.86</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>65%</t>
+          <t>80%</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2852,7 +2852,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>1,010원</t>
+          <t>1,009원</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2915,17 +2915,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Wed, 15 Jul 2026 01:48:25 GMT</t>
+          <t>Wed, 15 Jul 2026 13:45:57 GMT</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>연합인포맥스</t>
+          <t>연합뉴스</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>李대통령, MSCI 편입 불발 아쉬움…"국내 증시 안정화 도움될 텐데"</t>
+          <t>뉴욕증시, PPI 소화하며 상승 출발</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -2935,24 +2935,24 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTFA3MDEzcWxtWEtVbjAyRE1qUGtYLWNENmctUnBOdWlRSm10bm9STEF4bXFIUXk3eGdMYkI4MGdrZkZjNTFGb090SGlEQ01fckxtZng4ckpJay1hcUxvRGNxd1Jha0hvNzNyM0FzbVlMQjg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTFBNVmFmakpWM0V6dTFleWJHR1htTFVEQWJCZDhFSGVNTS0xVE15RUJMNGxrX094VXFHMVdPdHY5bGFRWXRfOFZua2ZwcU5rak9jRXhiNnYyQXFRbGfSAWBBVV95cUxPSnhjYlptN0ZMVUxrR0lGTWpxSGtCX1c3ejJMQWFkSzFKNTdWeXQ1SjQxbVlXTk9NX293OUhRMXpZdGx2aUg1MVc1dnRRM2psODNqMjEzVWpmZUZQU3QwbnE?oc=5</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Tue, 14 Jul 2026 07:48:01 GMT</t>
+          <t>Wed, 15 Jul 2026 12:31:47 GMT</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>머니투데이</t>
+          <t>대한민국 정책브리핑</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>주식시장 급락에 연기금 '줍줍'…어떤 종목을 샀을까 - 머니투데이</t>
+          <t>(설명) 매일경제(온라인), "노동법에 이미 기업 혼란 … '상설 노동자委' 서두를 일인가" 기사 관련</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -2962,78 +2962,78 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiaEFVX3lxTFBrNlgzb2ZIWU50V05sbVZUdnFCQ21NOUlkUElqVU5yQ2QzSXZpc0RtSkRlWTRCcS1Wb01YbXM2Rk9FLUplSUNaUUhYVWNKSTNmRHhaQUQwOXE4VGJSRk9NTkZPN01yWno10gFuQVVfeXFMTlNtU3FCUDg4ak5FMGVtSDZpeDVjUFJEUXgzWTRrc1lnWnVPOHpwTFo5bGZURzl0UlFnU0hiSmZmQ3U5dVd1bFMyb05MUDBLN1hpRUs5bThMY21uOU5IMUkwQzZMTUwxUXNEU09Na0E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTE9QOGlac21IaTRvSnl0MWVMTGRacHdBVExLYVh4WVQ0OUlINlN0cEdMZEI1elhER0czUkExM1R4amlYQk5JYm5tUGlLdUJTRjJwLTJPak05Z3VDSEpRVF9JN2c5SmlaQkdkNXZoSk1kSQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Tue, 14 Jul 2026 23:13:38 GMT</t>
+          <t>Wed, 15 Jul 2026 09:13:40 GMT</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>연합뉴스</t>
+          <t>연합인포맥스</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>[마켓뷰] 코스피, 美증시 훈풍에 최근 급락 만회하나</t>
+          <t>[중국증시-마감] 2022년 말 이후 최저 GDP에 하락</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>중립</t>
+          <t>부정적 (악재)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE9CdDA3MXU2SnJpaC13R0g2NHotRFJYdlFXLWV2RmtNOTFwQnpBeFA1bG41Zi1tS0xhYXl3VkJoRnY0eXBBaldtb2VfaXp4bm5lSHNsejVMTWU1STjSAWBBVV95cUxNTkJYcTNRdHZBLXRnUHl0MDI4Q19ycFF0dnNLMnNVR1Bxa2dBYTIzOWpsajg0Vldna3FRcXlMUGpzMkJuMXQ2aFJlaXBvNmd2Z3RPUnZKQUVkOWpGR2EzeC0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTFBxelJpWWx3YkNFVEsyY3J2QkF5SWFRZEtqQmJvYV9rLTFDajBZMkdUbFl4aHBvZ2t3SUNlTFgzUVI5T0NWRWUzdi1HYVI0VWtVcnRWbzR2b2tyZ0NzSEdESVZvUGQtOXBvTjFSYnlQQkk?oc=5</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tue, 14 Jul 2026 21:59:00 GMT</t>
+          <t>Wed, 15 Jul 2026 11:44:00 GMT</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>OhmyNews</t>
+          <t>경향신문</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>"곧 회복될 거야" 주식 하던 아내의 말수가 줄었습니다</t>
+          <t>미 증시에서 치솟은 하이닉스…투심도 살아나 7000피 탈환</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>긍정적 (호재)</t>
+          <t>중립</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5uWXFDSzhIdzR5M0szTWVlVlNGV0FhWkNGZnpadkRrUGJiV3NlVTlic0lUZWlVTS1MNUFFeU5VWU1SUzlMZzB2ZThrM3BRcFppcUZQLS1TcFRFUnJVc2xRRnhFTk5Od2E5b1l6a3RjamQ5eVdfd0ZV?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE1oMVBMaGNyLUlicHNSd1VTLTBMaEpxTmxpcm4wN3hKTnVZSDNRb0paeW4teDZMOFZhZkZPMldfNVNueTNBOWRzbFJTck5rWUs1ejNqeURRcktiQdIBX0FVX3lxTE9ZMmFQMUJ1RFlPTzJvVzFENEZtbVBkc1RWODdqdkFsR2JSTFNuMEl1UmNpZUp5VXRhdjdvelF1dUFsb2RsVDRrRDVVZEh4MkdaOUMwa29pNFFsUVNoQk00?oc=5</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Wed, 15 Jul 2026 02:25:39 GMT</t>
+          <t>Wed, 15 Jul 2026 05:48:00 GMT</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>대한민국 정책브리핑</t>
+          <t>동아일보</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>공주·부여·익산에 깃든 백제 역사를 거닐다…'2026 백제문화유산주간'</t>
+          <t>“주식 2억 벌었어” 친구 자랑에…뇌는 전치 4주 고통 느낀다</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -3043,51 +3043,51 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiakFVX3lxTE1peUVvdlRMVGlIanB3VU9EMVVyLUpnV3VYcTN3TEF3M0NVVXdqY3VmOE5UcjhBNS1EYkRUR1NkWDNYMUVXRm9sbHU1YkduRDZ0SWx0Q1MzQ0p4enVJNDJ4d0NPdWpRUjJMeFE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE8yc2VqTVoya25KYVZVOWhUWkR0YXIwZzQ1RGs5MmZ0NE8xUFVPRGcwdlpYaG94MmpNMkh3dUFQVjRWTy0yNlFlY0FILWZ0c1ZDVEJwRHdkTUk5UFBBZVdXSVdhUWg5VmkzMnh3UkZLcHpBdGxQSEHSAWZBVV95cUxNZE5BcnJSeVBwWXNibDAxMlYzcURjbkp0NmVmUWdZelZIWWtKOEU3RG5jTW9qam5KQVdlZ0NxVEctcXdWNXJGT1dWcHhDcXBQWFp5d3JuQng5SW8tNVE4dUVJSWFhSkE?oc=5</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Tue, 14 Jul 2026 22:58:00 GMT</t>
+          <t>Wed, 15 Jul 2026 09:00:00 GMT</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>경향신문</t>
+          <t>BBC</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>뉴욕증시, 물가우려 완화 속 반도체 랠리…SK하이닉스 ADR 27% 급등</t>
+          <t>'수출 호조에도 왜?' 중국 경제성장률 급락, 연간 목표치를 밑돌아</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>중립</t>
+          <t>긍정적 (호재)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE5FOHRpZ0h3cVRyRno2di1UVWk1alVOa3Y5Vk9WSkNjUzFRQUxNYng2aEd2ZnR3WG9xY0wtd0JVcDhkcnNUYUdac3U4ZXh4SkNCMHZ3QTJwc0NRUdIBX0FVX3lxTE9ZS3FIa0IzX3J3bEdyanFJdWFJWVF5Snl3TzZvMGNobWJjRi04SGpoOHVJVDNPc1IxQk52YlREdUE3MWhwanZhOXZ3dU1JR2tfVWxEMkNrQkhpeWVtcXRV?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiXEFVX3lxTE52UVRRTTIyQW5udGJFTjhSbEhmTHc4Q2QyTHdTd1BWNzE5b0p0U0hWZk5LbmNjdUY5ZWh2MlBZaEczSnd3RVZGSlRfLXlrdU9HYTlfdmthLW01dTVn0gFiQVVfeXFMUDU0UmVDOFl4VUpZYzlneGtDWHJCX3luT1pfdFhKaGZENGxvWTRjRTZYNTltalJDYXVBUG9IV3I2Qy1IMGljUEdDV0k3d3JQbmVXV05QUzNZSWl5QkJPQk1jV0E?oc=5</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Tue, 14 Jul 2026 08:59:35 GMT</t>
+          <t>Wed, 15 Jul 2026 07:11:00 GMT</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>매일경제</t>
+          <t>YTN</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>“주식이 이런거였어요?” 공포에 질린 주린이들…4조 던졌다</t>
+          <t>"역대급 주식 쏟아진다"...미 증시 강세장 끝물 신호?</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -3097,24 +3097,24 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiUkFVX3lxTFBYZWUxZ3dvZDQ0Znd2Z1MwLWJ2N2VoTDZ5aFZJMWdXZWh0ekJpV1o1WGtTUXVpX0Q4Nm5vMUlDOUIxdEhZNnl4Zmxrem9qQjZpZlE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiXkFVX3lxTE1uVHVMLUo3N25PNExvWVRFalhVRDlZWGhnclJvRURfT0ZOZ1NaZ0hjcURMQTR5NVh1Qzhscm1pWV9PUXFEbTYtRWhBX2xMay1rNWxiOVpveDVhY1hnRUE?oc=5</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Tue, 14 Jul 2026 22:43:31 GMT</t>
+          <t>Wed, 15 Jul 2026 11:00:02 GMT</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>MBC 뉴스</t>
+          <t>v.daum.net</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>증시, 이제 나아질까‥? 염승환 "다음 주가 중요 분기점" [모닝콜]</t>
+          <t>[경제칼럼] 압도적 성장의 길, 인천 경제 체질 바꿔야 한다</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -3124,24 +3124,24 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiekFVX3lxTE1aeHdmOGpidVI3eHR2b3oydVVJUTFHcVVxYW51dmdDY0RBbnlFcWtpelFoMEt6RHl0eTNhNTBiVGNfMkZoUUR5TXNFYk9oQ1FQMTB0UWVobDMzVWVpUEYzS0hwNzA0VVNmVzFyQ1pIY3lqVnVDM1d4bkR3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiT0FVX3lxTFBlRVNVeTR0RkF3U3NES0NfdXlQdlRwRks2bGJodlJJakZ6cW1yYzExLWVVVVlMby1Md3RrMDktY0pXOFpfVEZCREQ1d0J6ZWc?oc=5</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Wed, 15 Jul 2026 01:19:29 GMT</t>
+          <t>Wed, 15 Jul 2026 10:26:00 GMT</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>v.daum.net</t>
+          <t>KBS 뉴스</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>[김광석의 경제 읽어주는 남자] 금리보다 강력한 AI, 경제의 물길을 틀다</t>
+          <t>함명준 고성군수 “평화경제특구 1호 지정…경제 활력 되찾을 것”</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -3151,24 +3151,24 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiT0FVX3lxTE90c2JhR0dRZ2VXU056UDdvZDFKa1NxM0Y2UEZPTnA1NDNvV3BoRUd1a0wydVNRaEFsT192LXg2QWVGRnRBVkVOWEtPdHVaR3c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiZkFVX3lxTFBMSEo0djhqNV9XdUtqNktQMUNrT3BUWENCU0FZNlZDMU9HQlQzZ2lqSEQ0dkROdzZtYTFHMFFQSDVVM190Umx0VG1pMFNwZ2JmTEItaUZ0SmpjdkZlUHhaM092Vy1Ydw?oc=5</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Wed, 15 Jul 2026 01:52:39 GMT</t>
+          <t>Tue, 14 Jul 2026 07:48:01 GMT</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>수원시 인터넷신문</t>
+          <t>머니투데이</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>수원시도서관에서 책과 함께 알찬 여름방학 보내세요… 다채로운 독서문화 프로그램 운영</t>
+          <t>주식시장 급락에 연기금 '줍줍'…어떤 종목을 샀을까 - 머니투데이</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -3178,51 +3178,51 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiekFVX3lxTE1CSDNZSnNqMEppLXpxWWdwZXBzbnNqN1d2WkZickswSWdPS2FmUlJ2X0doaW5UcFBETjlfTEkxQmk1ZlZzVlEyUkpERHB0NFlkU21IdVNVdjRaZHo4UGhpbE96WjJhYTVDRDBzVkx4UWdWWkk3dEtfcUZB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiaEFVX3lxTFBrNlgzb2ZIWU50V05sbVZUdnFCQ21NOUlkUElqVU5yQ2QzSXZpc0RtSkRlWTRCcS1Wb01YbXM2Rk9FLUplSUNaUUhYVWNKSTNmRHhaQUQwOXE4VGJSRk9NTkZPN01yWno10gFuQVVfeXFMTlNtU3FCUDg4ak5FMGVtSDZpeDVjUFJEUXgzWTRrc1lnWnVPOHpwTFo5bGZURzl0UlFnU0hiSmZmQ3U5dVd1bFMyb05MUDBLN1hpRUs5bThMY21uOU5IMUkwQzZMTUwxUXNEU09Na0E?oc=5</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Wed, 15 Jul 2026 00:08:00 GMT</t>
+          <t>Wed, 15 Jul 2026 11:49:00 GMT</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>YTN</t>
+          <t>Investing.com 한국어</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>'롤러코스피' 강보합 마감...오늘 증시는?</t>
+          <t>InvestingPro, 이원다이애그노믹스 주식 54% 상승 어떻게 예측했나 By Investing.com</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>중립</t>
+          <t>긍정적 (호재)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiXkFVX3lxTE44bXRKUVlRY3diZDkxaVdXUVFoQkxVLUdsOUYxUVRfaGxJMlFBbVl6WHh4X3RVd0hPbVJROHZ2ODNUMzBjejJuQWppRms5NFVWLXVmVnVUSlBCS2RtYlE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFAtekV3RUFTUUM5d0JDcDVmcWFJc3U2cVh4eWkwQkpxZGZiZ1J5dXVzVDRneHBDWlhhQ2taS3RqbDFPT2Rwam1mNkxQMmNXRjRMc2h6eS1ZajZkVGl0S2hwRDdrRXc2V0J2RTRSSlRBNmxjU1pmR2c?oc=5</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Wed, 15 Jul 2026 02:00:00 GMT</t>
+          <t>Wed, 15 Jul 2026 02:09:31 GMT</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>한겨레</t>
+          <t>대한민국 정책브리핑</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>해외 투자은행들도 “삼전닉스 레버리지, 증시 변동성 초래 요인”</t>
+          <t>2026 하반기 경제성장전략 - 카드/한컷 | 멀티미디어</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -3232,24 +3232,24 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTE9pUmhLajJYajRHYlRUSGpyaHJ4cXU0OW4zYnJuR2pVT0ZUX3VNQU5oMWNseXVscERoMW5oTW54OUQ4czlZWGVVOENma1FrUEJVVW8wQVNMSUVSMjl3eWZOQlZPSXUyS1E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTE93YmNoay1MenRKY1VpckpwekkyMzdQd2Q1MEdnUkVJbVd1MFZkZWNJb2tfdGpQd19TeGhzcDdzaEFtUURmMXQtTGVlR053TmZ1bXR6TGVsdV9QQThnRmN2cmotcExXUURjUnFlR1pB?oc=5</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Wed, 15 Jul 2026 02:59:00 GMT</t>
+          <t>Wed, 15 Jul 2026 10:14:52 GMT</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>KBS 뉴스</t>
+          <t>연합인포맥스</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>‘문화가 있는 날’ 확대 결과…국민 10명 중 7명 “문화예술 활동 늘어”</t>
+          <t>[亞증시-종합] 예상 밑돈 GDP에 중국 홀로 약세</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -3259,24 +3259,24 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE8tT2w0TVBNTWwtRGVWaTRaLWNoRmlUZ1ZybzZRLVhWVWlLZlRKZGwzYm1YV3lkeEpMWjdZaW9nTDBJRVhVUTNCazZtWlVPNFp3dWFYVllfaTdxN28?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE5PWU9SVFNYOU5WRVJmSGEybzUyX2FWeXFJRlpuVjNPODQtVHVpTzNQZzBPRzhtR0FFQ1g4SG1rbXdRMVRxbjY2UGJEcnhIeUxBSEZZSjZJZjBYV2xfOGhtaHJuNk5VT0w3Rm1TeGpMNjg?oc=5</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Tue, 14 Jul 2026 20:49:21 GMT</t>
+          <t>Wed, 15 Jul 2026 08:00:00 GMT</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>연합인포맥스</t>
+          <t>YTN</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>[뉴욕증시] 한풀 꺾인 CPI에 안도 랠리…강세 마감</t>
+          <t>투자자 웃고 울리는 '도깨비 증시' 이대로 괜찮나</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -3286,68 +3286,68 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTFBXSS1fdm1xUXFFTnFKQW1DcWNEWDhzUHUtSjNZRUgtVWNBTXB5X1ZpN3RIS3dOR3BEVVkzMmZQSE9ISjU5aENnWWhkeXVfM3JyOXpJRXNYNnB5NGlNVk9BR1JMdzN6VWNUalpadk9lZE8?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiXkFVX3lxTE81MUk5NURuUzk1djBOTm5WSlE0czJmVlQwQm1xN3RyQkN6TzQ1bHFDY04yQndVY0xkWXk1eEZfbndzY3ZQUzE1WU1HNnp0UHJDY3NOdTE2UGlUNUJaYkE?oc=5</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Tue, 14 Jul 2026 20:45:58 GMT</t>
+          <t>Wed, 15 Jul 2026 07:35:39 GMT</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>연합뉴스</t>
+          <t>대한민국 정책브리핑</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>뉴욕증시, 물가우려 완화 속 반도체 랠리 재개…나스닥 1%↑(종합)</t>
+          <t>'문화요일' 확대 만족도 89.8%↑…10명 중 7명 "문화활동 늘어"</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>부정적 (악재)</t>
+          <t>중립</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE5TQ1pESF9fdE1UTTdLUUlJNkxRRlRhM3M0LTk2ZVduYjJaN3NQS3dxZFdieHBYM1NjRkRFUkVkZDZSQ2pmQ2hEcFJ4Y1RYV0NZZzUtY1dSYXZKWXfSAWBBVV95cUxNemhaTElKSVpZazh4bVRlNjc4Rms0bUNlQmlVZ2tWYkhGdGxFLWVUVnQwQ0Q4TmNsVWNZVmhkWk9fNGNickhuTDJEbnVyV2R6V1E4cnVZdVBzQ3Y0STdONnY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE5PM2c4bm02UUtTb01BTEF6UWFreHBWRTFkS3VJX29VeUhneWZ6SXRpd2x6TU9tV3lDYWowMExNUGVYVE14RjdiRHM5Qlo2Znp4ZUpyWFk2blA2QTh5ZVR3b2N2a0d2Z3p0UWcyLQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Wed, 15 Jul 2026 00:50:03 GMT</t>
+          <t>Wed, 15 Jul 2026 08:40:12 GMT</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>v.daum.net</t>
+          <t>연합인포맥스</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>[양기태의 글로벌 경제 읽기] 경제적 중력</t>
+          <t>[도쿄증시-마감] 반도체주 강세에 1%대 상승</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>중립</t>
+          <t>긍정적 (호재)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiT0FVX3lxTE1ieGljUFNBVmxWeHExZnV6SUk4ZzM4ZFpYMHE5Qno1SGkydVpISEZKeFY3RWF3aXg2MEpUY2xsMlFmN29pTVphYm95SFVicWs?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE9aRDU4ZXAxVmZaaWIySHAtMC1pdTFQeks2Q0Y4aUNpOTYwa2w5a0Y0Z251UUlzNWQzbVJvQ3JBdTctZ05TRTZiOWZIRmJhN09mWmlidzhjc1ZoVDdMUWRwLUk5dVJyeXJPOVFCd0J1enE?oc=5</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Wed, 15 Jul 2026 01:20:16 GMT</t>
+          <t>Wed, 15 Jul 2026 11:59:41 GMT</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3357,7 +3357,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>국세청 "상반기 물가·주식·부동산 탈세 6천200억 추징…철저히 조사"</t>
+          <t>모건스탠리, 2분기 순이익 사상 최대…주식 트레이딩 매출 69% '쑥'</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -3367,24 +3367,24 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE12YkJyeFlJU1NxcmJMcHBLeU9tY25HRUhzcVJYbFFuRVN2ckE2ZkxqS2l6Q0VISDFybWtMcjh2YVAtT1ZIWi01djNYWTJwb2VYYW5nWFhoV2FxM1VSbzBaUjdmMUVyOE5pVm9RUnN5MGI?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE9HejBoYzhkc1FXSTVUcm16ZXdYRmhYYnFQN0hQdGtESkRKQkdhOVhJQTZELUE2TzZURXB1b0tYcGNDbGNtNGowOEtfOGJER2dwUnFFTlJKU3Z1SkxKN2J2cTJyeE5WLWszTjZXd2NWSHI?oc=5</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Wed, 15 Jul 2026 02:16:57 GMT</t>
+          <t>Wed, 15 Jul 2026 04:10:47 GMT</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>v.daum.net</t>
+          <t>대한민국 정책브리핑</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>서울의 밤, 다시 깨어나다…서울시, '야간경제 활성화' 논의(종합)</t>
+          <t>K-푸드에 '테크' 날개 단다</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -3394,14 +3394,14 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiT0FVX3lxTE81UDRUTVJFTFNnTk5Ma1VJU1l6Z1VqYkZjNUFTZWU1Z3NHZmdPNzQwcFY2MjN5bWJXTG54VW5FZzZsZ3pWRlV6TzRGcEF5WHc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTFBsVGlZQTRON2thV0MtNkJ0UG1DUTNKMVp4RG54aTk5UzVnTXFyUFpxUnlfYngtTHFiVWZycGlDd2NmSEs5RmF4V2xicWp4TklWUkZkN3ViRjRGVUNYOENsOVhMNXVpdmVFSnBRXw?oc=5</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Wed, 15 Jul 2026 02:24:29 GMT</t>
+          <t>Mon, 13 Jul 2026 05:52:33 GMT</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3411,105 +3411,105 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>日 증시, 美 CPI 호재에 1%대 상승…닛케이 68,000선 회복</t>
+          <t>"반복되는 韓증시 급락 원인찾기"…레버리지·피로도·시클리컬 '삼중고'</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>긍정적 (호재)</t>
+          <t>중립</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE5SdmpVdmdNZFAyLVdRTVRuUTNJYU5iZ0NfakFoSW03cDUzby12a1ZmcUxMN1RjXzdFLVp3a2lSc1daa0RpdV92V2NjZ2RDSmlQbFdKeXRtcTVONEt4NXpNbE5IMmRuSTRIZC10aVQtMTk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE5ZTkM5bm1lZEY2MjRORHhKNDBNTzVYUEV6VHlBell6NEtINENOdnhxa0lUSVhxZ3pHaGkyLWRMLWs5ZTJXeHhGcXFIV2VWeUNoZnk3UEZQYmVxTjYzODJxbnJVUlZIUzBVa19hdFVvM1Q?oc=5</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Wed, 15 Jul 2026 00:12:12 GMT</t>
+          <t>Wed, 15 Jul 2026 06:52:38 GMT</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>v.daum.net</t>
+          <t>연합인포맥스</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>[친절한 경제] 흔들리는 반도체주 주가…너무 잘나가서 문제?</t>
+          <t>[증시-마감] 코스피, 美 물가 안도·반도체 랠리에 6.24% 급등</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>중립</t>
+          <t>긍정적 (호재)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiT0FVX3lxTE1DNFFJbkQzdnlyQzl6U3RQOTl0dDJhTXVSc0sxR0t1ZHZWQnRoaUl3enFFQW41cTlGX1gwM2UwamJlLXA4VkFsMkE0Q3hHQW8?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE1GWTRLZlhuVFZtWEFwS0JrOTNMRHRjQ3FKdFg3SlNDcmlxemUzcUpsS3NVWTZ2aDJJdEphejd5djh1Vk1rRkxEdTBzTEZ6UUJBcUZRcHMxYjBkdktMRVk5MmV1Vy1Oa1JOTkZwTzZIWHk?oc=5</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Wed, 15 Jul 2026 02:14:39 GMT</t>
+          <t>Wed, 15 Jul 2026 08:19:00 GMT</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>v.daum.net</t>
+          <t>연합뉴스TV</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>이재명 대통령 "국내 주식시장 불안한데, MSCI 왜 안 되나"</t>
+          <t>[시티&amp;로컬] 문화유산부터 첨단산업까지…"수원, 글로벌 관광도시로" 外</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>부정적 (악재)</t>
+          <t>중립</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiT0FVX3lxTFBUdXlEajhpZktnTEZhTWVha2ZCSTNZRmpwcGs2RzZNcEM1Q05QTFFuYWFPRFlaY0U4QzNKakp3cnlKbklMcjJIVFdNUHBFOHM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTE1vNnNIXzEwMlFsMGRlc2g3SW5jMHRWdXBGQWl4dXMtT3pWUXptTE9Pd3R1VGd2dUJKSXF4c1hEZVo3R2RPRWZiSzJ1N3FUOERGci1lRFhva1M0MjlMcDEtU0t4QXpFX3c?oc=5</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Tue, 14 Jul 2026 23:15:14 GMT</t>
+          <t>Wed, 15 Jul 2026 08:48:44 GMT</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>연합인포맥스</t>
+          <t>매일경제 마켓</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>크레이머 "AI 증시 과열 우려 과도…닷컴버블과는 거리 멀어"</t>
+          <t>'홀짝 증시' 언제까지…</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>부정적 (악재)</t>
+          <t>중립</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE5jY3RmVGtLTzEwQ2NISVJNcEFtYzA2cWQ1ZFNJTHBUd0tDNVBndDF4QVBodElvX2NVUTZtdFQzRFVUWU5NTEo5WV92VTlkQXJZTFFYbGlCRTZqX3Nra2JsbWpIQXZvQVY3VGRjYTlXeDU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiUkFVX3lxTE9ULURaelNncXNMV0NhUGM4X3lXLUl3bGppa3gtMGpYOGJyakpnay1La2g4RG9lTXNGckFJTzVVQU1lbFJIQlRUU3Z4Z1MtOWVEWWc?oc=5</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Mon, 13 Jul 2026 05:52:33 GMT</t>
+          <t>Wed, 15 Jul 2026 07:42:17 GMT</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3519,7 +3519,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>"반복되는 韓증시 급락 원인찾기"…레버리지·피로도·시클리컬 '삼중고'</t>
+          <t>남양유업, 기취득 자기주식 소각…220억원 규모</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -3529,24 +3529,24 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE5ZTkM5bm1lZEY2MjRORHhKNDBNTzVYUEV6VHlBell6NEtINENOdnhxa0lUSVhxZ3pHaGkyLWRMLWs5ZTJXeHhGcXFIV2VWeUNoZnk3UEZQYmVxTjYzODJxbnJVUlZIUzBVa19hdFVvM1Q?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE9fRHpfU3Ytd0lwWV9WeEpLLTBVcTYxXzZvWmllVUxWeXhyWlhZQmhPd3Q3SWZwbjVnZVpjbmw0UWthTURxcUJCVjJZUkstdlNjUEVrWlZZcFFmcnRudnNrSklwc081NFZnNlE1U2pfcVI?oc=5</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Wed, 15 Jul 2026 03:03:01 GMT</t>
+          <t>Wed, 15 Jul 2026 05:38:58 GMT</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>v.daum.net</t>
+          <t>연합뉴스</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>M2 통화량 석달째 증가…"주식 파생상품 늘어"</t>
+          <t>제주문화예술재단, 문화누리카드 전화결제 가맹점 모집</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -3556,24 +3556,24 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiT0FVX3lxTE81ZmE0c0JrWTcwWjZwdUtIRUpPZXNmT3l0UFhVQllSZ3VCbUJPLXJDX3ZjZnRpQXFsaUZWWVp1MDJNR0hPWUNyUzlidWZYSXc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTFAzdzZ5OUhfdElzZHp5Q1U3eTN5azZaR2ptdGJwNk0xTDN2MlBKUHdNMnFfMlZEMm9tdzVDOC01STNkOWpSTUN3US15OC0wSS0xdThSX1lsNTY4X0HSAWBBVV95cUxOckIxcmt5REJOR3pZME04LU84WlZDelYzXzNNLW1ieWJmM0hkUHFqbjFHbm5MbHpuQ3FEbWI2aGZyejVKTWp3NzhEaE1abmd6YzhoaEkzSTA1Zm9mNHJ3T00?oc=5</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Tue, 14 Jul 2026 23:01:51 GMT</t>
+          <t>Wed, 15 Jul 2026 12:03:39 GMT</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>연합인포맥스</t>
+          <t>매일경제 마켓</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>BofA "개별종목·지수 변동성 괴리 확대…증시 충격 위험 커져"</t>
+          <t>GLASS HOUSE BRANDS INC, 최대 1억 달러 규모 주식 발행 배포계약 개정</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -3583,24 +3583,24 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE03cU9hQjNlZTRVMEZQT0pHV3kzSkFDTWU3U1JCRHVjeDhtNkx5LTdYWTZ1VFg0UW1VZ3Y5Ymw2SmhFZ1JSR1hseHJ4b2xxbkNENzJjRng0T3k2NEZzdUpJbkJaUGVrYXlDNW9WVVVYb1U?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiUkFVX3lxTFB6bDdPUWI2b3MzT1E4NUlSOHVJLUV2N1BzQmthRXpwekxnaW9QVWRZUzE5QzZSUG13dmp2UlUwY2stWkk5RjB5ZFRtTzF3dk8zWHc?oc=5</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Wed, 15 Jul 2026 01:13:00 GMT</t>
+          <t>Wed, 15 Jul 2026 12:04:00 GMT</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>연합뉴스TV</t>
+          <t>YTN</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>[현장연결] 이 대통령, 국민참여 업무보고…경제분야 성과점검</t>
+          <t>"서울의 밤을 경제로"...새 성장동력 추진</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -3610,14 +3610,14 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTE1nQ0pndzF1RTlLYUhXTVRoVkQ3SlVsTlVnR0F6NHg4REVNZWtBMXI3TTh2Y0FYRVhvV1Z6Y1B0T2FBU3pyNlliSnBCRzlZZGxmcGZlSVF4ZjRRUTktRjJjTThKQnB4MXc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiXkFVX3lxTFBJNHlWNTNKNkdFNlgwSlFoWWJCY0tfWDhReXF5MGozUF85VFRaX0FQNVBYRkRrenBmd0dvWnZkbDQwNFZndkEtYmJVRXZKT244U1ZRSlYzWW40a1dOQ0E?oc=5</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Tue, 14 Jul 2026 22:59:27 GMT</t>
+          <t>Wed, 15 Jul 2026 08:24:00 GMT</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3627,7 +3627,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>[뉴욕마켓워치] CPI 호재 속 SK하이닉스 27% 폭등…주식·채권↑달러↓</t>
+          <t>토스, 첫 금융복합기업집단 지정…빅테크 첫 감독 대상</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -3637,14 +3637,14 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE9FZDdCSjNxRmtBcFJINF91UzlWc1Fia2EzQ0Vyd0JMQ1A2cExwWEVJbG5Ba1JjcDU3SHI4bDY3LUdaSGpEZkVNT3VuVXFyWWlPSW1EalFYakVpOVYwZW9TTHBCY05OSlRvcnpyNE01Yzc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE9TZXVvdVR5U2tQOUZhLUExUHRPQXg3ZTZJRV9yTjhBTFozdEFKSFE5SmhtamhCNklkcEthSmpWMGNueGtxeWlUOTJfSk5CcHJZcHljRDhRczB6ZDBJZWxHYWY0WUNmRDFYekhrdTFrZUXSAXRBVV95cUxQbjR1T0tncVIzOHRUNzdsd3pXc0JPTXVValNsT3g2Wmo0YndJa0xSbHdhcExrdUtLWTVjMzZOWXhPeVN4d0pCanVJejhkVWdmUFNDeWh2a2ZMSWJVSlI4TFNCR1FVRlk4dWVEcVVkR1lGQ3pEOQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Wed, 15 Jul 2026 01:54:04 GMT</t>
+          <t>Wed, 15 Jul 2026 06:55:52 GMT</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>오세훈, 민선 9기 첫 간부회의 주재…'야간경제 활성화' 논의</t>
+          <t>[르포]"주말 늦잠 대신 경제 공부"…2030 개미들의 '열혈' 투자 토론</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3664,24 +3664,24 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiT0FVX3lxTE5TTkpzMGxUaFpOcmNqX2NuZDBiY3pLOXVfY1dWSVRCRDhjN3BMVWtJaS1NUlhZZlBWNDFJSlFDdV91alNfQlR1bXhrVHctNk0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiT0FVX3lxTE1QalRFdHRza0xmQlZneUtqdTVQdkRRTUpLRS04X1RTY0tRREtBdFk0dnczZkJDQkJPdlMzTFhHVXItaG4zQVpRZlpySWVPcjQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Wed, 15 Jul 2026 01:21:00 GMT</t>
+          <t>Wed, 15 Jul 2026 10:07:33 GMT</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>knn.co.kr</t>
+          <t>매일경제 마켓</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>부산, 에이지테크 실증거점 조성사업 본격 착수</t>
+          <t>707 케이맨 홀딩스, 12대1 주식병합 단행..나스닥 상장 유지 목적</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -3691,24 +3691,24 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiVEFVX3lxTE1PYWFEWUxvUUhPeWFkYWk5MFExMmtVZExjcmRpSk9nQmJ5YUMyc3FhOHBsYVpyYi0tNjJGc2JMNGVxaWNzU1NTeER0WVh2X1p2aVBWNg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiUkFVX3lxTFB2OTFXUk9xX29xRzFNQWppdlJBc21UT2kzQlZnRy1feDlTWmpaQVgzc3EtWXhESkVXeWNFcUg2UjBybkNKbkhqQ2VSY3pyQzd0Ync?oc=5</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Wed, 15 Jul 2026 02:05:00 GMT</t>
+          <t>Wed, 15 Jul 2026 07:50:11 GMT</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>경향신문</t>
+          <t>연합뉴스</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>‘잠들지 않는 서울’ 만든다···야간경제 상생특구·달빛야장 본격추진</t>
+          <t>남양유업, 220억원 규모 자기주식 소각…"주주환원 활동 지속"</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE4tMl9JNjg4Z2kwb1M3NWhKaU9XMGdfWjA0dTNieV8tYzVadklkZzlRZFNENVJxclBoVlRTVmdLU0F5MUZodkdodVJtM3VUR1pPNXgxM0h0RTZ3d9IBX0FVX3lxTE4wYzRWTzBYMTVBeVdIaGl1ZGRpMGZ0ci1wMk1BQXZNdkR1b05zQjVHQ0tqVU5fTF92Q0xxVUZCdElqV25mNzBDZkJzQ0ZWNDhZRnB3VGdzUDVvMk91dFVN?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTFAwTzByMV84c05wUEhwdERRU05UMTlvd3gyQTRUTTh4UmFGRjVjMUwzUkxoQ3RhUUJRNTczWk9pZ0hqVWZLdXR5TC16alZyWHJIU1dkbDVyaTh0ajTSAWBBVV95cUxOYmp4TUUyUURidVpVN2UxWTNmMmpybGltN0JaU29adHBtbDZYQjZvNXZ4YVUzWlYzRVNnZ1MyZDNzVEtiNGNxUU1iNWtqZXVNSG40YVJ1Y1RpWnZWTTFPT0w?oc=5</t>
         </is>
       </c>
     </row>
@@ -3761,61 +3761,61 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AI/반도체 (기술)</t>
+          <t>결제/핀테크 (소비지표)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AI, 반도체</t>
+          <t>결제, 🛍️소비/매출폭발, 토스, 카드</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SK하이닉스, 한미반도체, 이수페타시스, 삼성전자</t>
+          <t>카카오페이, 네이버페이, KG이니시스, NHN KCP</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>80</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>정유/에너지 (원자재)</t>
+          <t>K-푸드/식품 (수출/소비)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>🔥유가상승수혜</t>
+          <t>수출, 🛍️소비/매출폭발</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>S-Oil, SK이노베이션, GS</t>
+          <t>삼양식품, CJ제일제당, 대상, 빙그레, 농심</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>원전/전력기기 (인프라)</t>
+          <t>여행/항공 (보복소비)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>🌱성수기/계절수혜</t>
+          <t>관광, 🌱성수기/계절수혜</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>LS일렉트릭, HD현대일렉트릭, 두산에너빌리티, 효성중공업</t>
+          <t>대한항공, 진에어, 제주항공, 하나투어, 모두투어, 호텔신라</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -3856,11 +3856,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6.56</v>
+        <v>6.43</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>한미반도체 (+27.71%)</t>
+          <t>한미반도체 (+29.88%)</t>
         </is>
       </c>
     </row>
@@ -3871,11 +3871,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4.75</v>
+        <v>3.48</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>삼성SDI (+8.07%)</t>
+          <t>에코프로비엠 (+7.37%)</t>
         </is>
       </c>
     </row>
@@ -3886,41 +3886,41 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2.99</v>
+        <v>3.12</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>삼성전자 (+7.22%)</t>
+          <t>LS일렉트릭 (+7.35%)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>배당/가치(안전)</t>
+          <t>기후/식량(방어)</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1.95</v>
+        <v>1.16</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>기아 (+4.3%)</t>
+          <t>시노펙스 (+3.18%)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>기후/식량(방어)</t>
+          <t>배당/가치(안전)</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1.42</v>
+        <v>1.1</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>시노펙스 (+3.57%)</t>
+          <t>기아 (+3.87%)</t>
         </is>
       </c>
     </row>
@@ -3931,41 +3931,41 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.32</v>
+        <v>0.05</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>TIGER 미국S&amp;P500 (+0.32%)</t>
+          <t>TIGER 미국S&amp;P500 (+0.05%)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>헷징/안전자산</t>
+          <t>신흥국(알파)</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-0.14</v>
+        <v>-0.28</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>TIGER 미국채10년선물 (-0.04%)</t>
+          <t>TIGER 인도니프티50 (-0.28%)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>신흥국(알파)</t>
+          <t>헷징/안전자산</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-0.28</v>
+        <v>-0.42</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>TIGER 인도니프티50 (-0.28%)</t>
+          <t>TIGER 미국채10년선물 (-0.34%)</t>
         </is>
       </c>
     </row>
@@ -4023,7 +4023,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>438,500원</t>
+          <t>434,000원</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -4032,7 +4032,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>32.8</v>
+        <v>34.2</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -4051,7 +4051,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2,143,000원</t>
+          <t>2,082,000원</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4060,7 +4060,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>29.4</v>
+        <v>33.2</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -4079,7 +4079,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>279,750원</t>
+          <t>288,500원</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -4088,7 +4088,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>27.3</v>
+        <v>23.5</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>

</xml_diff>